<commit_message>
Mise à jour de l'arbre 24/03/2026
</commit_message>
<xml_diff>
--- a/genealogie.xlsx
+++ b/genealogie.xlsx
@@ -245,6 +245,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -304,12 +305,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -439,440 +444,440 @@
   <dimension ref="A1:N14"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="10.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="10.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10.75"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="M2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N2" s="0" t="s">
+      <c r="N2" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="1" t="n">
+      <c r="I3" s="2" t="n">
         <v>10000</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M3" s="0" t="s">
+      <c r="M3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N3" s="0" t="s">
+      <c r="N3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>11000</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="M4" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>12000</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="0" t="s">
+      <c r="B5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>13000</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="2" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>14000</v>
       </c>
-      <c r="B7" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="0" t="s">
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="H7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="0" t="s">
+      <c r="M7" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>15000</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="0" t="s">
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>10000</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>10001</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>14001</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="H9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="1" t="n">
+      <c r="I9" s="2" t="n">
         <v>14000</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="K9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="M9" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>14100</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>14000</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <v>14001</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="H10" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>14200</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="B11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="1" t="n">
         <v>14000</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="1" t="n">
         <v>14001</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H11" s="0" t="s">
+      <c r="H11" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>14300</v>
       </c>
-      <c r="B12" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="0" t="n">
+      <c r="E12" s="1" t="n">
         <v>14000</v>
       </c>
-      <c r="F12" s="0" t="n">
+      <c r="F12" s="1" t="n">
         <v>14001</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="H12" s="1" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>14400</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="B13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E13" s="1" t="n">
         <v>14000</v>
       </c>
-      <c r="F13" s="0" t="n">
+      <c r="F13" s="1" t="n">
         <v>14001</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="2" t="n">
         <v>18095</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="H13" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>14201</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="G14" s="2" t="n">
         <v>19412</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="H14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I14" s="1" t="n">
+      <c r="I14" s="2" t="n">
         <v>14200</v>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>38770</v>
       </c>
-      <c r="K14" s="0" t="s">
+      <c r="K14" s="1" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>